<commit_message>
feat: Update HTML files and add new IPA and Projects pages with links and styling adjustments
</commit_message>
<xml_diff>
--- a/HTML/0 Excel SRC Files/Other E.xlsx
+++ b/HTML/0 Excel SRC Files/Other E.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Me\QuickAccessv2\HTML\0 Excel SRC Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A992883B-DD26-4AC5-A54C-B483FB9C8530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BFB1B9-DB57-4959-AC2F-958D836DE7B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="899" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="733">
   <si>
     <t>البيت الكبير</t>
   </si>
@@ -2569,6 +2569,9 @@
 اي ال main rules بتاعتي
 اي الحاجات إللي تنصحني أركز عليها
 هل ف احتمال يبقي فيه تعامل مع ال. Cloud</t>
+  </si>
+  <si>
+    <t>Math Is Fun</t>
   </si>
 </sst>
 </file>
@@ -4344,6 +4347,36 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4366,36 +4399,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="21" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5271,7 +5274,9 @@
       <c r="B3" s="201" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="118"/>
+      <c r="C3" s="200" t="s">
+        <v>732</v>
+      </c>
       <c r="D3" s="118"/>
       <c r="E3" s="200" t="s">
         <v>723</v>
@@ -5678,9 +5683,10 @@
     <hyperlink ref="H2" r:id="rId81" xr:uid="{969AC396-5B59-481C-A83A-7CF2FB12E437}"/>
     <hyperlink ref="G3" r:id="rId82" display="Quran" xr:uid="{1A09DF84-C826-4E70-AF94-16C57942C718}"/>
     <hyperlink ref="I5" r:id="rId83" xr:uid="{AE6A0070-D481-4725-8D96-23887A6B2F88}"/>
+    <hyperlink ref="C3" r:id="rId84" display="MathIsFun" xr:uid="{B35DD295-83A0-4BEF-85D2-E498D6EE24C0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId84"/>
+  <pageSetup orientation="portrait" r:id="rId85"/>
 </worksheet>
 </file>
 
@@ -8386,21 +8392,21 @@
       <c r="B1" s="143" t="s">
         <v>149</v>
       </c>
-      <c r="D1" s="223" t="s">
+      <c r="D1" s="215" t="s">
         <v>150</v>
       </c>
-      <c r="E1" s="224"/>
-      <c r="F1" s="211"/>
-      <c r="G1" s="215" t="s">
+      <c r="E1" s="216"/>
+      <c r="F1" s="221"/>
+      <c r="G1" s="225" t="s">
         <v>434</v>
       </c>
-      <c r="H1" s="216"/>
-      <c r="I1" s="211"/>
-      <c r="J1" s="219" t="s">
+      <c r="H1" s="226"/>
+      <c r="I1" s="221"/>
+      <c r="J1" s="211" t="s">
         <v>152</v>
       </c>
-      <c r="K1" s="220"/>
-      <c r="M1" s="217" t="s">
+      <c r="K1" s="212"/>
+      <c r="M1" s="209" t="s">
         <v>53</v>
       </c>
     </row>
@@ -8417,21 +8423,21 @@
       <c r="E2" s="121" t="s">
         <v>149</v>
       </c>
-      <c r="F2" s="211"/>
+      <c r="F2" s="221"/>
       <c r="G2" s="140" t="s">
         <v>153</v>
       </c>
       <c r="H2" s="141">
         <v>18</v>
       </c>
-      <c r="I2" s="211"/>
+      <c r="I2" s="221"/>
       <c r="J2" s="135" t="s">
         <v>409</v>
       </c>
       <c r="K2" s="136" t="s">
         <v>158</v>
       </c>
-      <c r="M2" s="218"/>
+      <c r="M2" s="210"/>
     </row>
     <row r="3" spans="1:13" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
@@ -8446,14 +8452,14 @@
       <c r="E3" s="12">
         <v>132</v>
       </c>
-      <c r="F3" s="211"/>
+      <c r="F3" s="221"/>
       <c r="G3" s="140" t="s">
         <v>156</v>
       </c>
       <c r="H3" s="141">
         <v>22</v>
       </c>
-      <c r="I3" s="211"/>
+      <c r="I3" s="221"/>
       <c r="J3" s="135" t="s">
         <v>163</v>
       </c>
@@ -8474,14 +8480,14 @@
       <c r="E4" s="12">
         <v>120</v>
       </c>
-      <c r="F4" s="211"/>
+      <c r="F4" s="221"/>
       <c r="G4" s="140" t="s">
         <v>160</v>
       </c>
       <c r="H4" s="141">
         <v>22</v>
       </c>
-      <c r="I4" s="211"/>
+      <c r="I4" s="221"/>
       <c r="J4" s="135" t="s">
         <v>486</v>
       </c>
@@ -8502,14 +8508,14 @@
       <c r="E5" s="13">
         <v>128</v>
       </c>
-      <c r="F5" s="211"/>
+      <c r="F5" s="221"/>
       <c r="G5" s="140" t="s">
         <v>168</v>
       </c>
       <c r="H5" s="141">
         <v>40</v>
       </c>
-      <c r="I5" s="211"/>
+      <c r="I5" s="221"/>
       <c r="J5" s="135" t="s">
         <v>171</v>
       </c>
@@ -8528,14 +8534,14 @@
       <c r="E6" s="13">
         <v>100</v>
       </c>
-      <c r="F6" s="211"/>
+      <c r="F6" s="221"/>
       <c r="G6" s="140" t="s">
         <v>169</v>
       </c>
       <c r="H6" s="141" t="s">
         <v>170</v>
       </c>
-      <c r="I6" s="211"/>
+      <c r="I6" s="221"/>
       <c r="J6" s="137" t="s">
         <v>453</v>
       </c>
@@ -8552,14 +8558,14 @@
         <v>439</v>
       </c>
       <c r="E7" s="13"/>
-      <c r="F7" s="211"/>
+      <c r="F7" s="221"/>
       <c r="G7" s="140" t="s">
         <v>443</v>
       </c>
       <c r="H7" s="141" t="s">
         <v>500</v>
       </c>
-      <c r="I7" s="211"/>
+      <c r="I7" s="221"/>
     </row>
     <row r="8" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
@@ -8572,16 +8578,16 @@
         <v>440</v>
       </c>
       <c r="E8" s="13"/>
-      <c r="F8" s="211"/>
+      <c r="F8" s="221"/>
       <c r="G8" s="140" t="s">
         <v>451</v>
       </c>
       <c r="H8" s="141"/>
-      <c r="I8" s="211"/>
-      <c r="J8" s="212" t="s">
+      <c r="I8" s="221"/>
+      <c r="J8" s="222" t="s">
         <v>458</v>
       </c>
-      <c r="K8" s="212"/>
+      <c r="K8" s="222"/>
     </row>
     <row r="9" spans="1:13" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
@@ -8594,14 +8600,14 @@
         <v>492</v>
       </c>
       <c r="E9" s="16"/>
-      <c r="F9" s="211"/>
+      <c r="F9" s="221"/>
       <c r="G9" s="140" t="s">
         <v>452</v>
       </c>
       <c r="H9" s="141" t="s">
         <v>499</v>
       </c>
-      <c r="I9" s="211"/>
+      <c r="I9" s="221"/>
       <c r="J9" s="127" t="s">
         <v>165</v>
       </c>
@@ -8616,14 +8622,14 @@
       <c r="E10" s="121" t="s">
         <v>149</v>
       </c>
-      <c r="F10" s="211"/>
+      <c r="F10" s="221"/>
       <c r="G10" s="140" t="s">
         <v>501</v>
       </c>
       <c r="H10" s="141" t="s">
         <v>502</v>
       </c>
-      <c r="I10" s="211"/>
+      <c r="I10" s="221"/>
       <c r="J10" s="127" t="s">
         <v>449</v>
       </c>
@@ -8644,8 +8650,8 @@
       <c r="E11" s="12">
         <v>143</v>
       </c>
-      <c r="F11" s="211"/>
-      <c r="I11" s="211"/>
+      <c r="F11" s="221"/>
+      <c r="I11" s="221"/>
       <c r="J11" s="127"/>
       <c r="K11" s="127"/>
     </row>
@@ -8656,12 +8662,12 @@
       <c r="B12" s="147"/>
       <c r="D12" s="15"/>
       <c r="E12" s="16"/>
-      <c r="F12" s="211"/>
-      <c r="G12" s="221" t="s">
+      <c r="F12" s="221"/>
+      <c r="G12" s="213" t="s">
         <v>151</v>
       </c>
-      <c r="H12" s="222"/>
-      <c r="I12" s="211"/>
+      <c r="H12" s="214"/>
+      <c r="I12" s="221"/>
       <c r="J12" s="127"/>
       <c r="K12" s="127"/>
     </row>
@@ -8678,14 +8684,14 @@
       <c r="E13" s="121" t="s">
         <v>149</v>
       </c>
-      <c r="F13" s="211"/>
+      <c r="F13" s="221"/>
       <c r="G13" s="132" t="s">
         <v>155</v>
       </c>
       <c r="H13" s="132" t="s">
         <v>157</v>
       </c>
-      <c r="I13" s="211"/>
+      <c r="I13" s="221"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="135" t="s">
@@ -8700,14 +8706,14 @@
       <c r="E14" s="12">
         <v>120</v>
       </c>
-      <c r="F14" s="211"/>
+      <c r="F14" s="221"/>
       <c r="G14" s="132" t="s">
         <v>162</v>
       </c>
       <c r="H14" s="132" t="s">
         <v>447</v>
       </c>
-      <c r="I14" s="211"/>
+      <c r="I14" s="221"/>
     </row>
     <row r="15" spans="1:13" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="150" t="s">
@@ -8718,14 +8724,14 @@
       </c>
       <c r="D15" s="15"/>
       <c r="E15" s="16"/>
-      <c r="F15" s="211"/>
+      <c r="F15" s="221"/>
       <c r="G15" s="132" t="s">
         <v>484</v>
       </c>
       <c r="H15" s="133" t="s">
         <v>454</v>
       </c>
-      <c r="I15" s="211"/>
+      <c r="I15" s="221"/>
       <c r="J15" s="105" t="s">
         <v>441</v>
       </c>
@@ -8740,14 +8746,14 @@
       <c r="B16" s="149" t="s">
         <v>176</v>
       </c>
-      <c r="F16" s="211"/>
+      <c r="F16" s="221"/>
       <c r="G16" s="132" t="s">
         <v>485</v>
       </c>
       <c r="H16" s="132" t="s">
         <v>482</v>
       </c>
-      <c r="I16" s="211"/>
+      <c r="I16" s="221"/>
       <c r="J16" s="105"/>
       <c r="K16" s="105"/>
     </row>
@@ -8764,14 +8770,14 @@
       <c r="E17" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="F17" s="211"/>
+      <c r="F17" s="221"/>
       <c r="G17" s="134" t="s">
         <v>487</v>
       </c>
       <c r="H17" s="134" t="s">
         <v>483</v>
       </c>
-      <c r="I17" s="211"/>
+      <c r="I17" s="221"/>
       <c r="J17" s="105"/>
       <c r="K17" s="105"/>
     </row>
@@ -8782,8 +8788,8 @@
       <c r="E18" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="F18" s="211"/>
-      <c r="I18" s="211"/>
+      <c r="F18" s="221"/>
+      <c r="I18" s="221"/>
     </row>
     <row r="19" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
@@ -8798,12 +8804,12 @@
       <c r="E19" s="28" t="s">
         <v>201</v>
       </c>
-      <c r="F19" s="211"/>
-      <c r="G19" s="213" t="s">
+      <c r="F19" s="221"/>
+      <c r="G19" s="223" t="s">
         <v>433</v>
       </c>
-      <c r="H19" s="214"/>
-      <c r="I19" s="211"/>
+      <c r="H19" s="224"/>
+      <c r="I19" s="221"/>
     </row>
     <row r="20" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="123" t="s">
@@ -8816,14 +8822,14 @@
       <c r="E20" s="28" t="s">
         <v>204</v>
       </c>
-      <c r="F20" s="211"/>
+      <c r="F20" s="221"/>
       <c r="G20" s="120" t="s">
         <v>178</v>
       </c>
       <c r="H20" s="68" t="s">
         <v>179</v>
       </c>
-      <c r="I20" s="211"/>
+      <c r="I20" s="221"/>
     </row>
     <row r="21" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="123" t="s">
@@ -8834,14 +8840,14 @@
         <v>497</v>
       </c>
       <c r="E21" s="28"/>
-      <c r="F21" s="211"/>
+      <c r="F21" s="221"/>
       <c r="G21" s="120" t="s">
         <v>437</v>
       </c>
       <c r="H21" s="68" t="s">
         <v>179</v>
       </c>
-      <c r="I21" s="211"/>
+      <c r="I21" s="221"/>
       <c r="J21" s="160"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -8853,10 +8859,10 @@
         <v>498</v>
       </c>
       <c r="E22" s="28"/>
-      <c r="F22" s="211"/>
+      <c r="F22" s="221"/>
       <c r="G22" s="120"/>
       <c r="H22" s="68"/>
-      <c r="I22" s="211"/>
+      <c r="I22" s="221"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="123" t="s">
@@ -8867,10 +8873,10 @@
         <v>190</v>
       </c>
       <c r="E23" s="28"/>
-      <c r="F23" s="211"/>
+      <c r="F23" s="221"/>
       <c r="G23" s="120"/>
       <c r="H23" s="68"/>
-      <c r="I23" s="211"/>
+      <c r="I23" s="221"/>
     </row>
     <row r="24" spans="1:11" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="123" t="s">
@@ -8883,12 +8889,12 @@
       <c r="E24" s="29" t="s">
         <v>205</v>
       </c>
-      <c r="F24" s="211"/>
+      <c r="F24" s="221"/>
       <c r="G24" s="139" t="s">
         <v>445</v>
       </c>
       <c r="H24" s="65"/>
-      <c r="I24" s="211"/>
+      <c r="I24" s="221"/>
     </row>
     <row r="25" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="123" t="s">
@@ -8924,10 +8930,10 @@
       </c>
     </row>
     <row r="30" spans="1:11" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="225" t="s">
+      <c r="A30" s="217" t="s">
         <v>180</v>
       </c>
-      <c r="B30" s="226"/>
+      <c r="B30" s="218"/>
       <c r="G30" s="131" t="s">
         <v>207</v>
       </c>
@@ -8996,24 +9002,24 @@
       <c r="B38" s="27"/>
     </row>
     <row r="39" spans="1:2" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="209" t="s">
+      <c r="A39" s="219" t="s">
         <v>202</v>
       </c>
-      <c r="B39" s="210"/>
+      <c r="B39" s="220"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="M1:M2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="A30:B30"/>
     <mergeCell ref="A39:B39"/>
     <mergeCell ref="I1:I24"/>
     <mergeCell ref="F1:F24"/>
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="G19:H19"/>
     <mergeCell ref="G1:H1"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A30:B30"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H30" location="Sports!A1" display="Sport" xr:uid="{0E60B1D8-A03B-425B-B677-F574292DD411}"/>

</xml_diff>